<commit_message>
旨辛チーズカレーを Extra Spicy Grilled Cheese Curry に
元のPDFは Spicy Grilled Cheese Curry で、補足に「定番と同名になるため
差別化が必要（例：Extra Spicy）」とあった。同名の相手は日本の定番ではなく
海外店のメニューで、Excelの備考に「別商品の可能性あり。要確認」と残っている。
2026年9月15日に松尾さんが Extra Spicy を選んだ。

補足の文面も「海外店の Spicy Grilled Cheese Curry と区別するため」に直した。
区分は「再販時に修正」のままなので、効くのは再販するときだけ。

ツール側（Supabase の nameEn）はまだ直していない。引き継ぎメモに残した。

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mamy2WdNr5xq9ik5Qc2QtW
</commit_message>
<xml_diff>
--- a/docs/rename-2026-10/out/商品名リネーム（2026年10月 全店改変）.xlsx
+++ b/docs/rename-2026-10/out/商品名リネーム（2026年10月 全店改変）.xlsx
@@ -2497,7 +2497,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Spicy Grilled Cheese Curry</t>
+          <t>Extra Spicy Grilled Cheese Curry</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2514,7 +2514,7 @@
       <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>過去限定。定番と同名になるため差別化が必要</t>
+          <t>過去限定。海外店の Spicy Grilled Cheese Curry と区別するため Extra Spicy を付けた（2026年9月15日 決定）</t>
         </is>
       </c>
     </row>

</xml_diff>